<commit_message>
feat: initializing database script and improving neo4j graph
</commit_message>
<xml_diff>
--- a/exports/excel_models/TSLA_Three_Statement_Model.xlsx
+++ b/exports/excel_models/TSLA_Three_Statement_Model.xlsx
@@ -565,7 +565,7 @@
         </is>
       </c>
       <c r="B4" s="5" t="n">
-        <v>88479262672.81</v>
+        <v>86877828054.3</v>
       </c>
       <c r="C4" s="5" t="n">
         <v>96000000000</v>
@@ -586,7 +586,7 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>48663594470.05</v>
+        <v>47782805429.87</v>
       </c>
       <c r="C5" s="5" t="n">
         <v>52800000000</v>
@@ -630,7 +630,7 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>17695852534.56</v>
+        <v>17375565610.86</v>
       </c>
       <c r="C7" s="5" t="n">
         <v>19200000000</v>
@@ -1072,10 +1072,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="36" customWidth="1" min="1" max="1"/>
+    <col width="37" customWidth="1" min="1" max="1"/>
     <col width="37" customWidth="1" min="2" max="2"/>
     <col width="20" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
@@ -1145,7 +1145,7 @@
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>Projected YoY Growth Rate (8.5%)</t>
+          <t>Projected YoY Growth Rate (10.5%)</t>
         </is>
       </c>
       <c r="B5" s="6" t="inlineStr">
@@ -1164,6 +1164,31 @@
       <c r="E5" s="14" t="inlineStr">
         <is>
           <t>Cross-referenced with consensus guidance RAG passages.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>TSLA Revenue verified</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>10-K</t>
+        </is>
+      </c>
+      <c r="C6" s="12" t="inlineStr">
+        <is>
+          <t>GROUNDED</t>
+        </is>
+      </c>
+      <c r="D6" s="13" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="E6" s="14" t="inlineStr">
+        <is>
+          <t>Audited by Verification Agent.</t>
         </is>
       </c>
     </row>

</xml_diff>